<commit_message>
rm useless slicename 9844a8a5bc532aa33e5d97a53377430e59928221
</commit_message>
<xml_diff>
--- a/ig/nr-review/StructureDefinition-as-practitionerrole.xlsx
+++ b/ig/nr-review/StructureDefinition-as-practitionerrole.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-05-16T08:18:01+00:00</t>
+    <t>2023-05-16T09:18:05+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -455,13 +455,13 @@
 </t>
   </si>
   <si>
-    <t>Autorité d'enregistrement représentant une institution (Ordre/ARS).</t>
+    <t>civiliteExercie + nomExercice + prenomExercice (ExerciceProfessionnel)</t>
   </si>
   <si>
     <t>Extension créée dans le cadre de l'Annuaire Santé pour définir l'identité d’exercice d’un professionnel.</t>
   </si>
   <si>
-    <t>Synonyme : AutoriteEnregistrement, Ordre</t>
+    <t>Concaténation des champs MOS : civilite + nomExercice + prenom</t>
   </si>
   <si>
     <t>PractitionerRole.extension:as-ext-practitionerrole-registration</t>
@@ -474,13 +474,13 @@
 </t>
   </si>
   <si>
-    <t>Eléments permettant de retrouver les informations d'inscription à un ordre par rapport à la profession de la personne physique sur une période et un département donné.</t>
+    <t>Autorité d'enregistrement représentant une institution (Ordre/ARS).</t>
   </si>
   <si>
     <t>Extension créée dans le cadre de l'Annuaire Santé pour prise en compte de la première inscription si "isFirst = true".</t>
   </si>
   <si>
-    <t>Synonymes RPPS : InscriptionOrdre</t>
+    <t>Synonyme : AutoriteEnregistrement, Ordre</t>
   </si>
   <si>
     <t>PractitionerRole.extension:as-ext-practitionerrole-education-level</t>
@@ -1359,7 +1359,7 @@
     <t>PractitionerRole.location</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(http://interopsante.org/fhir/StructureDefinition/FrLocation) &lt;&lt;contained&gt;&gt;
+    <t xml:space="preserve">Reference(http://interopsante.org/fhir/StructureDefinition/FrLocation)
 </t>
   </si>
   <si>

</xml_diff>